<commit_message>
add OpenSCAD roller prototypes and dimension truth policy
sync pulley/idler BOM specs and include validated STL exports
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -366,10 +366,10 @@
     <t>Strawberry Pets Store</t>
   </si>
   <si>
-    <t>MR85ZZ Ball Bearing (10pcs)</t>
-  </si>
-  <si>
-    <t>5x8x2.5mm MR85RS 10pcs blue seals</t>
+    <t>MR115ZZ Flanged Ball Bearing (10pcs)</t>
+  </si>
+  <si>
+    <t>5x11x4mm MR115ZZ flanged 10pcs</t>
   </si>
   <si>
     <t>8210696713585240</t>
@@ -381,7 +381,7 @@
     <t>Neoprene Rubber Gasket Strip</t>
   </si>
   <si>
-    <t>2000x15x3mm anti-vibration neoprene</t>
+    <t>2000x19x3mm neoprene belt strip target</t>
   </si>
   <si>
     <t>8210696713565240</t>
@@ -390,7 +390,7 @@
     <t>U Officer Store</t>
   </si>
   <si>
-    <t>2000x25x3mm anti-vibration neoprene</t>
+    <t>2000x19x3mm neoprene belt strip backup</t>
   </si>
   <si>
     <t>8210696713545240</t>

</xml_diff>